<commit_message>
updated repo, add base url for deploy at github
</commit_message>
<xml_diff>
--- a/public/examples/filled-shk-excel.xlsx
+++ b/public/examples/filled-shk-excel.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E1"/>
+  <dimension ref="A1:E45"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -416,9 +416,757 @@
         <v>test</v>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>2045522384557</v>
+      </c>
+      <c r="B2" t="str">
+        <v>20</v>
+      </c>
+      <c r="C2" t="str">
+        <v>WB_1601687241</v>
+      </c>
+      <c r="D2" t="str">
+        <v/>
+      </c>
+      <c r="E2" t="str">
+        <v>кол-во:20 row: к1 match: к1 count1:  rawType: к count2: 1</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>2045521734308</v>
+      </c>
+      <c r="B3" t="str">
+        <v>20</v>
+      </c>
+      <c r="C3" t="str">
+        <v>WB_1601687241</v>
+      </c>
+      <c r="D3" t="str">
+        <v/>
+      </c>
+      <c r="E3" t="str">
+        <v>кол-во:20 row: 20к1 match: 20к1 count1: 20 rawType: к count2: 1</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>2039468807300</v>
+      </c>
+      <c r="B4" t="str">
+        <v>10</v>
+      </c>
+      <c r="C4" t="str">
+        <v>WB_1601687240</v>
+      </c>
+      <c r="D4" t="str">
+        <v/>
+      </c>
+      <c r="E4" t="str">
+        <v>кол-во:20 row: 10к2 match: 10к2 count1: 10 rawType: к count2: 2</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>2039468807300</v>
+      </c>
+      <c r="B5" t="str">
+        <v>10</v>
+      </c>
+      <c r="C5" t="str">
+        <v>WB_1601687239</v>
+      </c>
+      <c r="D5" t="str">
+        <v/>
+      </c>
+      <c r="E5" t="str">
+        <v>кол-во:20 row: 10к3 match: 10к3 count1: 10 rawType: к count2: 3</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>2038719830555</v>
+      </c>
+      <c r="B6" t="str">
+        <v>10</v>
+      </c>
+      <c r="C6" t="str">
+        <v>WB_1601687239</v>
+      </c>
+      <c r="D6" t="str">
+        <v/>
+      </c>
+      <c r="E6" t="str">
+        <v>кол-во:20 row: 10к3-4 match: 10к3-4 count1: 10 rawType: к count2: 3-4</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>2038719830555</v>
+      </c>
+      <c r="B7" t="str">
+        <v>10</v>
+      </c>
+      <c r="C7" t="str">
+        <v>WB_1601687238</v>
+      </c>
+      <c r="D7" t="str">
+        <v/>
+      </c>
+      <c r="E7" t="str">
+        <v>кол-во:20 row: 10к3-4 match: 10к3-4 count1: 10 rawType: к count2: 3-4</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>2051268934154</v>
+      </c>
+      <c r="B8" t="str">
+        <v>16</v>
+      </c>
+      <c r="C8" t="str">
+        <v>WB_1601687237</v>
+      </c>
+      <c r="D8" t="str">
+        <v/>
+      </c>
+      <c r="E8" t="str">
+        <v>кол-во:60 row: 16к5 match: 16к5 count1: 16 rawType: к count2: 5</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>2051268934154</v>
+      </c>
+      <c r="B9" t="str">
+        <v>16</v>
+      </c>
+      <c r="C9" t="str">
+        <v>WB_1601687236</v>
+      </c>
+      <c r="D9" t="str">
+        <v/>
+      </c>
+      <c r="E9" t="str">
+        <v>кол-во:60 row: 16к6 match: 16к6 count1: 16 rawType: к count2: 6</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>2051268934154</v>
+      </c>
+      <c r="B10" t="str">
+        <v>16</v>
+      </c>
+      <c r="C10" t="str">
+        <v>WB_1601687235</v>
+      </c>
+      <c r="D10" t="str">
+        <v/>
+      </c>
+      <c r="E10" t="str">
+        <v>кол-во:60 row: 16к7 match: 16к7 count1: 16 rawType: к count2: 7</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>2051268934154</v>
+      </c>
+      <c r="B11" t="str">
+        <v>12</v>
+      </c>
+      <c r="C11" t="str">
+        <v>WB_1601687234</v>
+      </c>
+      <c r="D11" t="str">
+        <v/>
+      </c>
+      <c r="E11" t="str">
+        <v>кол-во:60 row: 12к8 match: 12к8 count1: 12 rawType: к count2: 8</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>2044452248540</v>
+      </c>
+      <c r="B12" t="str">
+        <v>16</v>
+      </c>
+      <c r="C12" t="str">
+        <v>WB_1601687237</v>
+      </c>
+      <c r="D12" t="str">
+        <v/>
+      </c>
+      <c r="E12" t="str">
+        <v>кол-во:60 row: 16к5 match: 16к5 count1: 16 rawType: к count2: 5</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>2044452248540</v>
+      </c>
+      <c r="B13" t="str">
+        <v>16</v>
+      </c>
+      <c r="C13" t="str">
+        <v>WB_1601687236</v>
+      </c>
+      <c r="D13" t="str">
+        <v/>
+      </c>
+      <c r="E13" t="str">
+        <v>кол-во:60 row: 16к6-7 match: 16к6-7 count1: 16 rawType: к count2: 6-7</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>2044452248540</v>
+      </c>
+      <c r="B14" t="str">
+        <v>16</v>
+      </c>
+      <c r="C14" t="str">
+        <v>WB_1601687235</v>
+      </c>
+      <c r="D14" t="str">
+        <v/>
+      </c>
+      <c r="E14" t="str">
+        <v>кол-во:60 row: 16к6-7 match: 16к6-7 count1: 16 rawType: к count2: 6-7</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>2044452248540</v>
+      </c>
+      <c r="B15" t="str">
+        <v>12</v>
+      </c>
+      <c r="C15" t="str">
+        <v>WB_1601687234</v>
+      </c>
+      <c r="D15" t="str">
+        <v/>
+      </c>
+      <c r="E15" t="str">
+        <v>кол-во:60 row: 12к8 match: 12к8 count1: 12 rawType: к count2: 8</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>2051738226116</v>
+      </c>
+      <c r="B16" t="str">
+        <v>88</v>
+      </c>
+      <c r="C16" t="str">
+        <v>WB_1601687233</v>
+      </c>
+      <c r="D16" t="str">
+        <v/>
+      </c>
+      <c r="E16" t="str">
+        <v xml:space="preserve">кол-во:88 row: м match: м count1:  rawType: м count2: </v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>2046885966756</v>
+      </c>
+      <c r="B17" t="str">
+        <v>10</v>
+      </c>
+      <c r="C17" t="str">
+        <v>WB_1601687232</v>
+      </c>
+      <c r="D17" t="str">
+        <v/>
+      </c>
+      <c r="E17" t="str">
+        <v xml:space="preserve">кол-во:50 row: 10м match: 10м count1: 10 rawType: м count2: </v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>2046885966756</v>
+      </c>
+      <c r="B18" t="str">
+        <v>10</v>
+      </c>
+      <c r="C18" t="str">
+        <v>WB_1601687231</v>
+      </c>
+      <c r="D18" t="str">
+        <v/>
+      </c>
+      <c r="E18" t="str">
+        <v xml:space="preserve">кол-во:50 row: 10м match: 10м count1: 10 rawType: м count2: </v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>2046885966756</v>
+      </c>
+      <c r="B19" t="str">
+        <v>10</v>
+      </c>
+      <c r="C19" t="str">
+        <v>WB_1601687230</v>
+      </c>
+      <c r="D19" t="str">
+        <v/>
+      </c>
+      <c r="E19" t="str">
+        <v xml:space="preserve">кол-во:50 row: 10м match: 10м count1: 10 rawType: м count2: </v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>2046885966756</v>
+      </c>
+      <c r="B20" t="str">
+        <v>10</v>
+      </c>
+      <c r="C20" t="str">
+        <v>WB_1601687229</v>
+      </c>
+      <c r="D20" t="str">
+        <v/>
+      </c>
+      <c r="E20" t="str">
+        <v xml:space="preserve">кол-во:50 row: 10м match: 10м count1: 10 rawType: м count2: </v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>2046885966756</v>
+      </c>
+      <c r="B21" t="str">
+        <v>10</v>
+      </c>
+      <c r="C21" t="str">
+        <v>WB_1601687228</v>
+      </c>
+      <c r="D21" t="str">
+        <v/>
+      </c>
+      <c r="E21" t="str">
+        <v xml:space="preserve">кол-во:50 row: 10м match: 10м count1: 10 rawType: м count2: </v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="str">
+        <v>2045104087272</v>
+      </c>
+      <c r="B22" t="str">
+        <v>10</v>
+      </c>
+      <c r="C22" t="str">
+        <v>WB_1601687227</v>
+      </c>
+      <c r="D22" t="str">
+        <v/>
+      </c>
+      <c r="E22" t="str">
+        <v>кол-во:60 row: 10к9-10 match: 10к9-10 count1: 10 rawType: к count2: 9-10</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="str">
+        <v>2045104087272</v>
+      </c>
+      <c r="B23" t="str">
+        <v>10</v>
+      </c>
+      <c r="C23" t="str">
+        <v>WB_1601687226</v>
+      </c>
+      <c r="D23" t="str">
+        <v/>
+      </c>
+      <c r="E23" t="str">
+        <v>кол-во:60 row: 10к9-10 match: 10к9-10 count1: 10 rawType: к count2: 9-10</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="str">
+        <v>2045921869037</v>
+      </c>
+      <c r="B24" t="str">
+        <v>10</v>
+      </c>
+      <c r="C24" t="str">
+        <v>WB_1601687225</v>
+      </c>
+      <c r="D24" t="str">
+        <v/>
+      </c>
+      <c r="E24" t="str">
+        <v>кол-во:60 row: 10к98 match: 10к98 count1: 10 rawType: к count2: 98</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="str">
+        <v>2045921869037</v>
+      </c>
+      <c r="B25" t="str">
+        <v>10</v>
+      </c>
+      <c r="C25" t="str">
+        <v>WB_1601687224</v>
+      </c>
+      <c r="D25" t="str">
+        <v/>
+      </c>
+      <c r="E25" t="str">
+        <v>кол-во:60 row: 10к99 match: 10к99 count1: 10 rawType: к count2: 99</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="str">
+        <v>2045921869037</v>
+      </c>
+      <c r="B26" t="str">
+        <v>10</v>
+      </c>
+      <c r="C26" t="str">
+        <v>WB_1601687223</v>
+      </c>
+      <c r="D26" t="str">
+        <v/>
+      </c>
+      <c r="E26" t="str">
+        <v xml:space="preserve">кол-во:60 row: 10м match: 10м count1: 10 rawType: м count2: </v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="str">
+        <v>2045921869037</v>
+      </c>
+      <c r="B27" t="str">
+        <v>10</v>
+      </c>
+      <c r="C27" t="str">
+        <v>WB_1601687222</v>
+      </c>
+      <c r="D27" t="str">
+        <v/>
+      </c>
+      <c r="E27" t="str">
+        <v xml:space="preserve">кол-во:60 row: 10м match: 10м count1: 10 rawType: м count2: </v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="str">
+        <v>2045921869037</v>
+      </c>
+      <c r="B28" t="str">
+        <v>10</v>
+      </c>
+      <c r="C28" t="str">
+        <v>WB_1601687221</v>
+      </c>
+      <c r="D28" t="str">
+        <v/>
+      </c>
+      <c r="E28" t="str">
+        <v xml:space="preserve">кол-во:60 row: 10м match: 10м count1: 10 rawType: м count2: </v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="str">
+        <v>2045921869037</v>
+      </c>
+      <c r="B29" t="str">
+        <v>10</v>
+      </c>
+      <c r="C29" t="str">
+        <v>WB_1601687220</v>
+      </c>
+      <c r="D29" t="str">
+        <v/>
+      </c>
+      <c r="E29" t="str">
+        <v xml:space="preserve">кол-во:60 row: 10м match: 10м count1: 10 rawType: м count2: </v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="str">
+        <v>2046124235353</v>
+      </c>
+      <c r="B30" t="str">
+        <v>8</v>
+      </c>
+      <c r="C30" t="str">
+        <v>WB_1601687227</v>
+      </c>
+      <c r="D30" t="str">
+        <v/>
+      </c>
+      <c r="E30" t="str">
+        <v>кол-во:40 row: 8к9-16 match: 8к9-16 count1: 8 rawType: к count2: 9-16</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="str">
+        <v>2046124235353</v>
+      </c>
+      <c r="B31" t="str">
+        <v>8</v>
+      </c>
+      <c r="C31" t="str">
+        <v>WB_1601687226</v>
+      </c>
+      <c r="D31" t="str">
+        <v/>
+      </c>
+      <c r="E31" t="str">
+        <v>кол-во:40 row: 8к9-16 match: 8к9-16 count1: 8 rawType: к count2: 9-16</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="str">
+        <v>2046124235353</v>
+      </c>
+      <c r="B32" t="str">
+        <v>8</v>
+      </c>
+      <c r="C32" t="str">
+        <v>WB_1601687219</v>
+      </c>
+      <c r="D32" t="str">
+        <v/>
+      </c>
+      <c r="E32" t="str">
+        <v>кол-во:40 row: 8к9-16 match: 8к9-16 count1: 8 rawType: к count2: 9-16</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="str">
+        <v>2046124235353</v>
+      </c>
+      <c r="B33" t="str">
+        <v>8</v>
+      </c>
+      <c r="C33" t="str">
+        <v>WB_1601687218</v>
+      </c>
+      <c r="D33" t="str">
+        <v/>
+      </c>
+      <c r="E33" t="str">
+        <v>кол-во:40 row: 8к9-16 match: 8к9-16 count1: 8 rawType: к count2: 9-16</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="str">
+        <v>2046124235353</v>
+      </c>
+      <c r="B34" t="str">
+        <v>8</v>
+      </c>
+      <c r="C34" t="str">
+        <v>WB_1601687217</v>
+      </c>
+      <c r="D34" t="str">
+        <v/>
+      </c>
+      <c r="E34" t="str">
+        <v>кол-во:40 row: 8к9-16 match: 8к9-16 count1: 8 rawType: к count2: 9-16</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="str">
+        <v>2046124235353</v>
+      </c>
+      <c r="B35" t="str">
+        <v>8</v>
+      </c>
+      <c r="C35" t="str">
+        <v>WB_1601687216</v>
+      </c>
+      <c r="D35" t="str">
+        <v/>
+      </c>
+      <c r="E35" t="str">
+        <v>кол-во:40 row: 8к9-16 match: 8к9-16 count1: 8 rawType: к count2: 9-16</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="str">
+        <v>2046124235353</v>
+      </c>
+      <c r="B36" t="str">
+        <v>8</v>
+      </c>
+      <c r="C36" t="str">
+        <v>WB_1601687215</v>
+      </c>
+      <c r="D36" t="str">
+        <v/>
+      </c>
+      <c r="E36" t="str">
+        <v>кол-во:40 row: 8к9-16 match: 8к9-16 count1: 8 rawType: к count2: 9-16</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="str">
+        <v>2046124235353</v>
+      </c>
+      <c r="B37" t="str">
+        <v>8</v>
+      </c>
+      <c r="C37" t="str">
+        <v>WB_1601687214</v>
+      </c>
+      <c r="D37" t="str">
+        <v/>
+      </c>
+      <c r="E37" t="str">
+        <v>кол-во:40 row: 8к9-16 match: 8к9-16 count1: 8 rawType: к count2: 9-16</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="str">
+        <v>2045045285140</v>
+      </c>
+      <c r="B38" t="str">
+        <v>8</v>
+      </c>
+      <c r="C38" t="str">
+        <v>WB_1601687227</v>
+      </c>
+      <c r="D38" t="str">
+        <v/>
+      </c>
+      <c r="E38" t="str">
+        <v>кол-во:40 row: 8к9 match: 8к9 count1: 8 rawType: к count2: 9</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="str">
+        <v>2045045285140</v>
+      </c>
+      <c r="B39" t="str">
+        <v>8</v>
+      </c>
+      <c r="C39" t="str">
+        <v>WB_1601687226</v>
+      </c>
+      <c r="D39" t="str">
+        <v/>
+      </c>
+      <c r="E39" t="str">
+        <v>кол-во:40 row: 8к10 match: 8к10 count1: 8 rawType: к count2: 10</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="str">
+        <v>2045045285140</v>
+      </c>
+      <c r="B40" t="str">
+        <v>8</v>
+      </c>
+      <c r="C40" t="str">
+        <v>WB_1601687219</v>
+      </c>
+      <c r="D40" t="str">
+        <v/>
+      </c>
+      <c r="E40" t="str">
+        <v>кол-во:40 row: 8к11 match: 8к11 count1: 8 rawType: к count2: 11</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="str">
+        <v>2045045285140</v>
+      </c>
+      <c r="B41" t="str">
+        <v>8</v>
+      </c>
+      <c r="C41" t="str">
+        <v>WB_1601687218</v>
+      </c>
+      <c r="D41" t="str">
+        <v/>
+      </c>
+      <c r="E41" t="str">
+        <v>кол-во:40 row: 8к12 match: 8к12 count1: 8 rawType: к count2: 12</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="str">
+        <v>2045045285140</v>
+      </c>
+      <c r="B42" t="str">
+        <v>8</v>
+      </c>
+      <c r="C42" t="str">
+        <v>WB_1601687217</v>
+      </c>
+      <c r="D42" t="str">
+        <v/>
+      </c>
+      <c r="E42" t="str">
+        <v>кол-во:40 row: 8к13 match: 8к13 count1: 8 rawType: к count2: 13</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="str">
+        <v>2045045285140</v>
+      </c>
+      <c r="B43" t="str">
+        <v>8</v>
+      </c>
+      <c r="C43" t="str">
+        <v>WB_1601687216</v>
+      </c>
+      <c r="D43" t="str">
+        <v/>
+      </c>
+      <c r="E43" t="str">
+        <v>кол-во:40 row: 8к14 match: 8к14 count1: 8 rawType: к count2: 14</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="str">
+        <v>2045045285140</v>
+      </c>
+      <c r="B44" t="str">
+        <v>8</v>
+      </c>
+      <c r="C44" t="str">
+        <v>WB_1601687215</v>
+      </c>
+      <c r="D44" t="str">
+        <v/>
+      </c>
+      <c r="E44" t="str">
+        <v>кол-во:40 row: 8к15 match: 8к15 count1: 8 rawType: к count2: 15</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="str">
+        <v>2045045285140</v>
+      </c>
+      <c r="B45" t="str">
+        <v>8</v>
+      </c>
+      <c r="C45" t="str">
+        <v>WB_1601687214</v>
+      </c>
+      <c r="D45" t="str">
+        <v/>
+      </c>
+      <c r="E45" t="str">
+        <v>кол-во:40 row: 8к16 match: 8к16 count1: 8 rawType: к count2: 16</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E1"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E45"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>